<commit_message>
feat: Integrate HealthBeauty web and mobile with shared API
Ship the admin web and customer Flutter app in one repository with a shared API.
Include account administration, role permissions, audit logs, responsive pages,
linked Staff account creation and booking/billing contract fixes.

Revoke rotated or discarded refresh sessions correctly on both clients.
Allow localhost development clients for Chrome testing and document clone/setup.
Keep machine secrets, build output, caches and legacy handoff notes out of Git.
Update the API catalog to distinguish implemented operations from planned routes.

Validate fresh source installs: API 182 tests, web 35 tests, mobile 52 tests;
web lint/build and Flutter analyze/web/Android debug builds pass.

BREAKING CHANGE: POST /api/v1/staff requires email and password for a Staff login.

Co-authored-by: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/KLCN021_API_Catalog.xlsx
+++ b/KLCN021_API_Catalog.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conventions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Catalog'!$A$1:$I$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Catalog'!$A$1:$J$126</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -79,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -89,6 +89,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -454,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" style="4" min="1" max="1"/>
@@ -466,6 +469,7 @@
     <col width="38" customWidth="1" style="4" min="7" max="7"/>
     <col width="30" customWidth="1" style="4" min="8" max="8"/>
     <col width="32" customWidth="1" style="4" min="9" max="9"/>
+    <col width="36" customWidth="1" style="4" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="4">
@@ -514,6 +518,11 @@
           <t>Mã lỗi/Ghi chú</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Trạng thái triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -559,6 +568,11 @@
           <t>409 email đã tồn tại</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -604,6 +618,11 @@
           <t>All failures logged; default5 wrong passwords lock15min. Config Authentication:MaxFailedAttempts/LockoutMinutes. Unauthorized401.</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -649,6 +668,11 @@
           <t>Inactive or temporarily locked account401.</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -694,6 +718,11 @@
           <t>Only caller-owned refresh token revoked.</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -735,6 +764,11 @@
         </is>
       </c>
       <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -776,6 +810,11 @@
         </is>
       </c>
       <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -817,6 +856,11 @@
         </is>
       </c>
       <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -858,6 +902,11 @@
         </is>
       </c>
       <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -899,6 +948,11 @@
         </is>
       </c>
       <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -940,6 +994,11 @@
         </is>
       </c>
       <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -985,6 +1044,11 @@
           <t>404 không tồn tại</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1030,6 +1094,11 @@
           <t>409 đang được sử dụng</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1052,7 +1121,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>List staff for customer booking</t>
+          <t>Nhân viên cho quản trị và chọn lịch</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1067,12 +1136,17 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[{ nhanVienId, hoTen, chucVu, chuyenMon, soDienThoai, ngayVaoLam }]</t>
+          <t>[{nhanVienId,hoTen,chucVu,chuyenMon,soDienThoai,ngayVaoLam,taiKhoanId}]</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Authenticated; GET access expanded only. Writes/schedules remain Admin/Manager.</t>
+          <t>taiKhoanId chỉ cho quản trị, Customer nhận null; không trả mật khẩu.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
         </is>
       </c>
     </row>
@@ -1097,25 +1171,34 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Tạo nhân viên</t>
+          <t>Tạo nhân viên kèm tài khoản Staff</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>STAFF.WRITE</t>
+          <t>Admin/Manager/Reception + STAFF.WRITE</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>hoTen, chucVu, chuyenMon, soDienThoai</t>
+          <t>fullName, position?, specialty?, phone?, hireDate?, email, password (8–128)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>NhanVienDto</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="n"/>
+          <t>201 {nhanVienId,taiKhoanId,hoTen,chucVu,chuyenMon,soDienThoai,ngayVaoLam}</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Transaction account+employee+audit; hash password; 400 dữ liệu sai, 409 email trùng.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1161,6 +1244,11 @@
           <t>Finite detail projection; no EF back references. 404 missing.</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1183,25 +1271,34 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật nhân viên</t>
+          <t>Sửa hồ sơ nhân viên</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>STAFF.WRITE</t>
+          <t>Admin/Manager/Reception + STAFF.WRITE</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>NhanVien fields</t>
+          <t>fullName, position?, specialty?, phone?, hireDate?</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>NhanVienDto</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="n"/>
+          <t>Employee fields</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Không thay đổi thông tin đăng nhập.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1247,6 +1344,11 @@
           <t>409 if any appointment/schedule references staff, including cancelled history.</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1288,6 +1390,11 @@
         </is>
       </c>
       <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1333,6 +1440,11 @@
           <t>409 trùng ca</t>
         </is>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1374,6 +1486,11 @@
         </is>
       </c>
       <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1415,6 +1532,11 @@
         </is>
       </c>
       <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1456,6 +1578,11 @@
         </is>
       </c>
       <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1497,6 +1624,11 @@
         </is>
       </c>
       <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1538,6 +1670,11 @@
         </is>
       </c>
       <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1579,6 +1716,11 @@
         </is>
       </c>
       <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1620,6 +1762,11 @@
         </is>
       </c>
       <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1661,6 +1808,11 @@
         </is>
       </c>
       <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1702,6 +1854,11 @@
         </is>
       </c>
       <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1743,6 +1900,11 @@
         </is>
       </c>
       <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1784,6 +1946,11 @@
         </is>
       </c>
       <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="25" customHeight="1" s="4">
       <c r="A32" s="2" t="n">
@@ -1825,6 +1992,11 @@
         </is>
       </c>
       <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1866,6 +2038,11 @@
         </is>
       </c>
       <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1907,6 +2084,11 @@
         </is>
       </c>
       <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1948,6 +2130,11 @@
         </is>
       </c>
       <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1989,6 +2176,11 @@
         </is>
       </c>
       <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2030,6 +2222,11 @@
         </is>
       </c>
       <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2071,6 +2268,11 @@
         </is>
       </c>
       <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2112,6 +2314,11 @@
         </is>
       </c>
       <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2153,6 +2360,11 @@
         </is>
       </c>
       <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2198,6 +2410,11 @@
           <t>Individual candidate slots every30minutes; full duration must fit shift and avoid busy intervals; service duration overrides durationMinutes. Alias available-slots. 400 invalid input.</t>
         </is>
       </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2243,6 +2460,11 @@
           <t>Catalog-derived expectedPrice; complete active combo composition/date required. Management also APPOINTMENT.WRITE. Invalid service/combo/shift400; overlap409.</t>
         </is>
       </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2288,6 +2510,11 @@
           <t>Management APPOINTMENT.READ sees all; Staff APPOINTMENT.READ assigned only; Customer own records.</t>
         </is>
       </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2333,6 +2560,11 @@
           <t>403 other customer; 404 missing; no EF back references.</t>
         </is>
       </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2378,6 +2610,11 @@
           <t>409 chuyển trạng thái không hợp lệ</t>
         </is>
       </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2419,6 +2656,11 @@
         </is>
       </c>
       <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2464,6 +2706,11 @@
           <t>409 unless pending/confirmed or if intervals overlap; 400 invalid time/staff or outside selected staff shift.</t>
         </is>
       </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2509,6 +2756,11 @@
           <t>204 only for ChoXacNhan/DaXacNhan/DaDen. 409 otherwise; 403 other customer; 404 missing.</t>
         </is>
       </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2554,6 +2806,11 @@
           <t>Completed/matching booked lines required. Whole redeemed points clamp to actual discount; ledger references invoice. Management also INVOICE.WRITE.</t>
         </is>
       </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2599,6 +2856,11 @@
           <t>Staff see all; customer own only.</t>
         </is>
       </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2640,6 +2902,11 @@
         </is>
       </c>
       <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2681,6 +2948,11 @@
         </is>
       </c>
       <c r="I52" s="2" t="n"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2722,6 +2994,11 @@
         </is>
       </c>
       <c r="I53" s="2" t="n"/>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2767,6 +3044,11 @@
           <t>Customer403; repeated409; zero-total settles without payment row or earned points.</t>
         </is>
       </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2808,6 +3090,11 @@
         </is>
       </c>
       <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2849,6 +3136,11 @@
         </is>
       </c>
       <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2890,6 +3182,11 @@
         </is>
       </c>
       <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2931,6 +3228,11 @@
         </is>
       </c>
       <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -2976,6 +3278,11 @@
           <t>discountType: PhanTram (0..100) or SoTien (&gt;=0); normalized; valid date interval required.</t>
         </is>
       </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3017,6 +3324,11 @@
         </is>
       </c>
       <c r="I60" s="2" t="n"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3058,6 +3370,11 @@
         </is>
       </c>
       <c r="I61" s="2" t="n"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="25" customHeight="1" s="4">
       <c r="A62" s="2" t="n">
@@ -3099,6 +3416,11 @@
         </is>
       </c>
       <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3144,6 +3466,11 @@
           <t>Same validation as create: normalized unique code, valid promotion/customer, future expiry, nonnegative amount. 400 invalid;409 duplicate.</t>
         </is>
       </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3185,6 +3512,11 @@
         </is>
       </c>
       <c r="I64" s="2" t="n"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3226,6 +3558,11 @@
         </is>
       </c>
       <c r="I65" s="2" t="n"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3267,6 +3604,11 @@
         </is>
       </c>
       <c r="I66" s="2" t="n"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3308,6 +3650,11 @@
         </is>
       </c>
       <c r="I67" s="2" t="n"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3349,6 +3696,11 @@
         </is>
       </c>
       <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3390,6 +3742,11 @@
         </is>
       </c>
       <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3431,6 +3788,11 @@
         </is>
       </c>
       <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3472,6 +3834,11 @@
         </is>
       </c>
       <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -3513,6 +3880,11 @@
         </is>
       </c>
       <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3554,6 +3926,11 @@
         </is>
       </c>
       <c r="I73" s="2" t="n"/>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3595,6 +3972,11 @@
         </is>
       </c>
       <c r="I74" s="2" t="n"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3636,6 +4018,11 @@
         </is>
       </c>
       <c r="I75" s="2" t="n"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3677,6 +4064,11 @@
         </is>
       </c>
       <c r="I76" s="2" t="n"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -3718,6 +4110,11 @@
         </is>
       </c>
       <c r="I77" s="2" t="n"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -3759,6 +4156,11 @@
         </is>
       </c>
       <c r="I78" s="2" t="n"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -3804,6 +4206,11 @@
           <t>state không hợp lệ: 400</t>
         </is>
       </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3845,6 +4252,11 @@
         </is>
       </c>
       <c r="I80" s="2" t="n"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -3890,6 +4302,11 @@
           <t>Không cho hủy liên kết cuối cùng</t>
         </is>
       </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -3935,6 +4352,11 @@
           <t>Nên giới hạn Admin/Security</t>
         </is>
       </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -3976,6 +4398,11 @@
         </is>
       </c>
       <c r="I83" s="2" t="n"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -4017,6 +4444,11 @@
         </is>
       </c>
       <c r="I84" s="2" t="n"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4058,6 +4490,11 @@
         </is>
       </c>
       <c r="I85" s="2" t="n"/>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có trong Swagger hiện tại</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -4103,144 +4540,2014 @@
           <t>403 wrong owner; 400 invalid time/staff or outside selected shift; 404 missing; 409 unless pending/confirmed or interval overlap.</t>
         </is>
       </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="5" t="inlineStr">
         <is>
           <t>Staff</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="5" t="inlineStr">
         <is>
           <t>/api/v1/staff/me/appointments</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E87" s="5" t="inlineStr">
         <is>
           <t>Own assigned appointments</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F87" s="5" t="inlineStr">
         <is>
           <t>Staff + APPOINTMENT.READ</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
+      <c r="G87" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="H87" s="5" t="inlineStr">
         <is>
           <t>Array of assigned appointment summaries</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>Staff profile missing returns []; no other employee records.</t>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>403 nếu chưa có hồ sơ; chỉ dữ liệu được phân công cho hồ sơ liên kết tài khoản.</t>
+        </is>
+      </c>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="n">
+      <c r="A88" s="5" t="n">
         <v>87</v>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>Staff</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="5" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="5" t="inlineStr">
         <is>
           <t>/api/v1/staff/me/schedules</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="E88" s="5" t="inlineStr">
         <is>
           <t>Own work schedules</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="F88" s="5" t="inlineStr">
         <is>
           <t>Staff + STAFF.READ</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr">
+      <c r="G88" s="5" t="inlineStr">
         <is>
           <t>from?, to?</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="H88" s="5" t="inlineStr">
         <is>
           <t>Array of own schedule summaries</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>Staff profile missing returns []; no other employee records.</t>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>403 nếu chưa có hồ sơ; chỉ dữ liệu được phân công cho hồ sơ liên kết tài khoản.</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
+      <c r="A89" s="5" t="n">
         <v>88</v>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="5" t="inlineStr">
         <is>
           <t>Reviews</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="5" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" s="5" t="inlineStr">
         <is>
           <t>/api/v1/reviews/pending</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E89" s="5" t="inlineStr">
         <is>
           <t>Reviews awaiting moderation</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F89" s="5" t="inlineStr">
         <is>
           <t>Admin/Manager + REVIEW.MODERATE</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
+      <c r="G89" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="H89" s="5" t="inlineStr">
         <is>
           <t>Review summary[] (latest200)</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr">
+      <c r="I89" s="5" t="inlineStr">
         <is>
           <t>Public GET reviews remains visible reviews only.</t>
         </is>
       </c>
+      <c r="J89" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Accounts</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/accounts</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Tạo tài khoản và hồ sơ liên kết</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Admin + ACCOUNT.WRITE</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>email, password, fullName, phone?, roleId, staffId?</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>201 AdminAccountResponse</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>staffId chỉ cho Staff; 409 email hoặc hồ sơ đã có tài khoản.</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Accounts</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/accounts/{id}/role</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>Gán vai trò/liên kết nhân viên</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Admin + ACCOUNT.WRITE</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>roleId, staffId?</t>
+        </is>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>200 AdminAccountResponse</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>Giữ role Staff và đổi hồ sơ cũ chưa có lịch/ca; giữ lịch của hồ sơ chọn, revoke refresh và audit.</t>
+        </is>
+      </c>
+      <c r="J91" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/auth/permissions</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>Quyền hiện tại của tài khoản</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Authenticated</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>{role,permissions[]}</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>Chỉ quyền được cấp và đang hoạt động trong database.</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Combos</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/combos/{id}</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Promotions</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/promotions/vouchers/{id}</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Promotions</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/promotions/{id}</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J95" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/service-categories/{id}</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J96" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>StaffManagement</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/staff/schedules/{id}</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J97" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/accounts</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>; query: keyword?</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J98" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/audit-logs</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>; query: take?</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J99" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/login-logs</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>; query: take?</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I100" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J100" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/permissions</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J101" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/roles</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J102" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/roles/{roleId}/permissions</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J103" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>AppointmentManagement</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/appointments/available-slots</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>; query: date?, staffId?, serviceId?, durationMinutes?</t>
+        </is>
+      </c>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I104" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J104" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Combos</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/combos</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J105" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Combos</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/combos/{id}</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J106" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/customers/me</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I107" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J107" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/customers/me/points</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I108" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J108" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>CustomerVouchers</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/customers/me/vouchers</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I109" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J109" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/staff/schedules</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>; query: staffId?, from?, to?</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I110" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J110" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>StaffManagement</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/staff/{id}/appointments</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I111" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J111" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Promotions</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/vouchers</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>; query: keyword?, active?</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I112" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J112" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/accounts/{accountId}/status</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>; query: active?</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>AppointmentManagement</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/appointments/{id}/status</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>body: AppointmentStatusRequest</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I114" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J114" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Promotions</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/promotions/vouchers/{id}/status</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>; query: active?</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I115" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J115" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/reviews/{id}/moderation</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>; query: visible?</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I116" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J116" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Combos</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/combos</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>body: ComboRequest</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I117" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J117" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>Promotions</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/promotions/vouchers</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>body: VoucherRequest</t>
+        </is>
+      </c>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I118" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J118" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Promotions</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/promotions/vouchers/validate</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>; query: code?</t>
+        </is>
+      </c>
+      <c r="H119" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I119" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J119" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/reviews/invoices/{invoiceId}</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G120" s="5" t="inlineStr">
+        <is>
+          <t>body: ReviewRequest</t>
+        </is>
+      </c>
+      <c r="H120" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I120" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J120" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/staff/schedules</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>body: WorkScheduleRequest</t>
+        </is>
+      </c>
+      <c r="H121" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I121" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J121" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/roles/{roleId}/permissions/{permissionId}</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>body: RolePermissionRequest</t>
+        </is>
+      </c>
+      <c r="H122" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I122" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J122" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Combos</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/combos/{id}</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>body: ComboRequest</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I123" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J123" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/customers/me</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>body: UpdateCustomerRequest</t>
+        </is>
+      </c>
+      <c r="H124" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I124" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J124" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Promotions</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/promotions/vouchers/{id}</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>body: VoucherRequest</t>
+        </is>
+      </c>
+      <c r="H125" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I125" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J125" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>StaffManagement</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>/api/v1/staff/schedules/{id}</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint triển khai trong Swagger</t>
+        </is>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>body: WorkScheduleRequest</t>
+        </is>
+      </c>
+      <c r="H126" s="5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I126" s="5" t="inlineStr">
+        <is>
+          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+        </is>
+      </c>
+      <c r="J126" s="5" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I86"/>
+  <autoFilter ref="A1:J126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(api): Add password recovery reviews and notifications
Add email OTP password recovery with session revocation, service review
summaries and appointment review metadata, and a durable notification inbox
with Firebase delivery. Keep broadcast read state scoped to each account
and protect appointment and invoice changes against concurrent updates.

Include repeatable SQL upgrades 04 through 06 and Vietnamese integration
instructions for the web and Flutter maintainers. Preserve client sources
and keep machine credentials and local feedback outside version control.

Validate with 281 API tests and isolated SQL concurrency and rollback checks.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/KLCN021_API_Catalog.xlsx
+++ b/KLCN021_API_Catalog.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conventions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Catalog'!$A$1:$J$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Catalog'!$A$1:$J$133</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" style="4" min="1" max="1"/>
@@ -776,7 +776,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Yêu cầu đặt lại mật khẩu</t>
+          <t>Yêu cầu OTP khôi phục mật khẩu</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Anonymous + IP rate limit</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -806,13 +806,17 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>204 No Content</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n"/>
+          <t>200 {message}; không trả debugOtp</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Generic cho email tồn tại/không tồn tại; OTP15phút, gửi lại60giây,5lần/giờ/tài khoản; IP10lần/10phút.</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Chưa có trong Swagger hiện tại</t>
+          <t>Đã triển khai</t>
         </is>
       </c>
     </row>
@@ -2502,12 +2506,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>{ items: AppointmentResponse[], totalCount, page, pageSize }</t>
+          <t>{items:AppointmentResponse[],totalCount,page,pageSize}; items add invoiceId,invoiceStatus,hasReviewed,reviewStars</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Management APPOINTMENT.READ sees all; Staff APPOINTMENT.READ assigned only; Customer own records.</t>
+          <t>Management APPOINTMENT.READ sees all; Staff APPOINTMENT.READ assigned only; Customer own records. Latest invoice by date/ID descending; hidden review still reviewed. Missing invoice: null metadata, false reviewed.</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3544,20 +3548,24 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Public/Admin</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>serviceId?, rating?, page, size</t>
+          <t>serviceId? (positive integer)</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>PagedResult&lt;DanhGiaDto&gt;</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="n"/>
+          <t>{averageRating, totalReviews, items:[{danhGiaId,hoaDonId,soSao,binhLuan,ngayDanhGia,tenKhachHang}]}</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Visible only; direct/combo services. Full-set statistics, max200 recent items. Empty average0. Response changed from array: clients read items.</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
           <t>Đã triển khai</t>
@@ -3631,28 +3639,32 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Danh sách thông báo</t>
+          <t>Hộp thư thông báo của khách hàng</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Authenticated</t>
+          <t>Authenticated account with customer profile</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>unreadOnly, page, size</t>
+          <t>page=1,pageSize=20(max100),unreadOnly=false</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>PagedResult&lt;ThongBaoDto&gt;</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="n"/>
+          <t>200 {items:[{id,title,body,type,data,isRead,createdAt}],totalCount,unreadCount,page,pageSize}</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Own private + broadcasts; per-account read state; data is JSON string; UTC timestamp. Missing auth401; no customer403. Requires migration06.</t>
+        </is>
+      </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>Chưa có trong Swagger hiện tại</t>
+          <t>Đã triển khai</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4684,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Admin/Manager + REVIEW.MODERATE</t>
+          <t>Admin/Manager/Reception + REVIEW.MODERATE</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -6022,22 +6034,22 @@
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+          <t>Admin/Manager/Reception + REVIEW.MODERATE</t>
         </is>
       </c>
       <c r="G116" s="5" t="inlineStr">
         <is>
-          <t>; query: visible?</t>
+          <t>query visible (boolean)</t>
         </is>
       </c>
       <c r="H116" s="5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204 No Content</t>
         </is>
       </c>
       <c r="I116" s="5" t="inlineStr">
         <is>
-          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+          <t>false=An, true=HienThi; 404 missing review.</t>
         </is>
       </c>
       <c r="J116" s="5" t="inlineStr">
@@ -6217,27 +6229,27 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>Endpoint triển khai trong Swagger</t>
+          <t>Review owned paid invoice; visible immediately</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>Theo vai trò, quyền và phạm vi dữ liệu tại API</t>
+          <t>Authenticated customer, invoice owner</t>
         </is>
       </c>
       <c r="G120" s="5" t="inlineStr">
         <is>
-          <t>body: ReviewRequest</t>
+          <t>stars (1..5), comment? (max1000)</t>
         </is>
       </c>
       <c r="H120" s="5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201 {danhGiaId,hoaDonId,soSao,binhLuan,trangThai,ngayDanhGia}</t>
         </is>
       </c>
       <c r="I120" s="5" t="inlineStr">
         <is>
-          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+          <t>HienThi by default; unpaid400, not owner404, duplicate409 including concurrent requests. Requires migration05.</t>
         </is>
       </c>
       <c r="J120" s="5" t="inlineStr">
@@ -6546,8 +6558,358 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>/api/v1/auth/reset-password</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Xác nhận OTP và đặt mật khẩu mới</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Anonymous + IP rate limit</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>email, otp (chuỗi6số), newPassword (8–128)</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>200 {message}; không tự đăng nhập</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>OTP1lần/5lượt thử;400sai/hết hạn/đã dùng;429IP20lần/10phút; resetSecurityStamp+revokeallrefresh+audit.</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>/api/v1/reviews/appointments/{appointmentId}</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Review owned completed appointment</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Authenticated customer, appointment owner</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>stars (1..5), comment? (max1000)</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>201 review summary; HienThi</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Latest invoice must be paid; invalid/incomplete/unpaid400, not owner404, duplicate409. Same uniqueness as invoice route.</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/device-token</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Đăng ký hoặc cập nhật token FCM</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Authenticated account with customer profile</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>{token (max500,no whitespace),deviceType:android|ios|web}</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>200 {message}</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Token unique and case-sensitive; rebind to current account/customer. Invalid400. Missing auth401; no customer403. Requires migration06.</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/device-token</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Hủy token trước khi đăng xuất</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Authenticated account with customer profile</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>query token (URL encoded)</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Owner-qualified update; idempotent; cannot disable token rebound to another account. Missing auth401; no customer403. Requires migration06.</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/unread-count</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Đếm thông báo chưa đọc</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Authenticated account with customer profile</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>200 {unreadCount}</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Counts own private and global notifications; independent per account. Missing auth401; no customer403. Requires migration06.</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/{id}/read</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Đánh dấu một thông báo đã đọc</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Authenticated account with customer profile</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Own inbox only; inaccessible404; duplicate read idempotent. Missing auth401; no customer403. Requires migration06.</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>/api/v1/notifications/read-all</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Đánh dấu hộp thư hiện tại đã đọc</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Authenticated account with customer profile</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Per-account receipt snapshot; other customers unaffected. Missing auth401; no customer403. Requires migration06.</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J126"/>
+  <autoFilter ref="A1:J133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6558,7 +6920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18" customWidth="1" style="4" min="1" max="1"/>
@@ -6886,6 +7248,57 @@
       <c r="C19" s="2" t="inlineStr">
         <is>
           <t>POST/GET appointment list; decimal money is retained. Detail/reschedule still use existing entity-shaped JSON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DeviceTokenRequest</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>token, deviceType</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>POST /notifications/device-token</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NotificationResponse</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>id,title,body,type,data:string?,isRead,createdAt UTC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GET /notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ThongBaoDaDoc</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>thongBaoId,taiKhoanId,ngayDoc (composite key)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Per-account read receipts; shared broadcast remains unread for other customers</t>
         </is>
       </c>
     </row>
@@ -6900,7 +7313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="13" customWidth="1" style="4" min="1" max="1"/>
@@ -7053,6 +7466,18 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Notifications (2026-10-17)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06migration adds3tables + appointment/invoice rowversion; total28business tables. Durable push outbox; Firebase default disabled; per-account broadcast reads. Vietnamese handoff REVIEWS.md section11.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(api): Add media loyalty review and reporting integration
Add durable reminders, point voucher exchange, persisted review management and XLSX reports.

Provide additive database migrations and a Vietnamese handoff for the Web team.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/KLCN021_API_Catalog.xlsx
+++ b/KLCN021_API_Catalog.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conventions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Catalog'!$A$1:$J$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Catalog'!$A$1:$J$136</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J133"/>
+  <dimension ref="A1:J144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" style="4" min="1" max="1"/>
@@ -1747,28 +1747,32 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Xem điểm thưởng/lịch sử điểm</t>
+          <t>Lịch sử điểm của khách cho quản trị</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Admin/Reception/Owner</t>
+          <t>Admin/Manager/Reception + CUSTOMER.READ</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>page, size</t>
+          <t>page=1,pageSize=20(1..100)</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>PointBalance + giaoDichDiem[]</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="n"/>
+          <t>{customerId,diemThuong,transactions,totalCount,page,pageSize}</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Transactions include invoiceId/voucherId links;404 missing;400 invalidpagination.</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Chưa có trong Swagger hiện tại</t>
+          <t>Đã triển khai</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1950,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>PagedResult&lt;DichVuDto&gt;</t>
+          <t>PagedResult&lt;DichVuDto&gt;; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I31" s="2" t="n"/>
@@ -1987,12 +1991,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>loaiDichVuId, tenDichVu, gia, thoiLuong, moTa</t>
+          <t>loaiDichVuId, tenDichVu, gia, thoiLuong, moTa; imageUrl? (HTTP/S,max2048; update null preserves, empty clears)</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>DichVuDto</t>
+          <t>DichVuDto; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I32" s="2" t="n"/>
@@ -2038,7 +2042,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>DichVuDetailDto</t>
+          <t>DichVuDetailDto; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I33" s="2" t="n"/>
@@ -2079,12 +2083,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>DichVu fields</t>
+          <t>DichVu fields; imageUrl? (HTTP/S,max2048; update null preserves, empty clears)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>DichVuDto</t>
+          <t>DichVuDto; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I34" s="2" t="n"/>
@@ -2807,7 +2811,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Completed/matching booked lines required. Whole redeemed points clamp to actual discount; ledger references invoice. Management also INVOICE.WRITE.</t>
+          <t>Completed/matching booked lines required. Whole redeemed points clamp to actual discount; ledger references invoice. Management also INVOICE.WRITE. Unique perappointment; customer/voucherconcurrency409; unclaimedpointvoucher400.</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3558,12 +3562,12 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>{averageRating, totalReviews, items:[{danhGiaId,hoaDonId,soSao,binhLuan,ngayDanhGia,tenKhachHang}]}</t>
+          <t>{averageRating,totalReviews,items:[{danhGiaId,hoaDonId,soSao,binhLuan,ngayDanhGia,tenKhachHang,reply,repliedAt}]}</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Visible only; direct/combo services. Full-set statistics, max200 recent items. Empty average0. Response changed from array: clients read items.</t>
+          <t>Visible non-deleted reviews only; full-set statistics, max200 latest. Read items envelope. Reply author account remains private. Requires SQL11.</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3735,28 +3739,32 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Báo cáo lịch hẹn</t>
+          <t>Legacy appointment status totals</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>REPORT.READ + existing role allowlist</t>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>from, to, groupBy, status?</t>
+          <t>from?,to? (inclusive/exclusive)</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>ReportResult</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="n"/>
+          <t>[{status,count}]</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Backward-compatible status totals; use appointment-summary for day/week/month.</t>
+        </is>
+      </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>Đã triển khai</t>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -3781,28 +3789,32 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Báo cáo doanh thu</t>
+          <t>Legacy paid invoice summary</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>REPORT.READ + existing role allowlist</t>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>from, to, groupBy, type?</t>
+          <t>from?,to? (inclusive/exclusive)</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>RevenueReport</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="n"/>
+          <t>{invoiceCount,revenue}</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Paid invoices only by invoice creation date; use order-summary for time periods.</t>
+        </is>
+      </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>Đã triển khai</t>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -3827,28 +3839,32 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Báo cáo khách hàng</t>
+          <t>Legacy top customers</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>REPORT.READ + existing role allowlist</t>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>from, to, segment?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>CustomerReport</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="n"/>
+          <t>CustomerReport[] (max200)</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Not a total customer count or new-customer report. Use new-customers.</t>
+        </is>
+      </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Đã triển khai</t>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -3873,28 +3889,32 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Báo cáo dịch vụ/combo/nhân viên</t>
+          <t>Legacy paid service/combo sales</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>REPORT.READ + existing role allowlist</t>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>from, to, serviceId?, staffId?</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>ServiceReport</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="n"/>
+          <t>[{dichVuId,name,quantity,revenue}]</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>All-time paid gross line sales. Combo identity distinct internally, legacy response shape retained. Use order-breakdown for explicit IDs and filters.</t>
+        </is>
+      </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>Đã triển khai</t>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -3919,28 +3939,32 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Xuất báo cáo Excel/PDF</t>
+          <t>Export report as genuine Excel XLSX</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>REPORT.READ + existing role allowlist</t>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>reportType, from, to, format</t>
+          <t>report=appointments|orders|breakdown|new-customers; report filters</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>File stream</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="n"/>
+          <t>XLSX file</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>REPORT.READ. Max10000 rows including metadata; filter before export. Orders export is time summary. PDF via existing Web browser print only; no PDF API. SQL12 prepared, not applied locally: SSPI blocked live verification.</t>
+        </is>
+      </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Chưa có trong Swagger hiện tại</t>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -5494,7 +5518,7 @@
       </c>
       <c r="H105" s="5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I105" s="5" t="inlineStr">
@@ -5544,7 +5568,7 @@
       </c>
       <c r="H106" s="5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I106" s="5" t="inlineStr">
@@ -6049,7 +6073,7 @@
       </c>
       <c r="I116" s="5" t="inlineStr">
         <is>
-          <t>false=An, true=HienThi; 404 missing review.</t>
+          <t>false=An, true=HienThi. Deleted/missing404; concurrent change409. REVIEW.MODERATE; SQL11.</t>
         </is>
       </c>
       <c r="J116" s="5" t="inlineStr">
@@ -6089,12 +6113,12 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>body: ComboRequest</t>
+          <t>body: ComboRequest; imageUrl? (HTTP/S,max2048; update null preserves, empty clears)</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I117" s="5" t="inlineStr">
@@ -6139,7 +6163,7 @@
       </c>
       <c r="G118" s="5" t="inlineStr">
         <is>
-          <t>body: VoucherRequest</t>
+          <t>body: VoucherRequest; pointsCost=0 (0..1000000)</t>
         </is>
       </c>
       <c r="H118" s="5" t="inlineStr">
@@ -6149,7 +6173,7 @@
       </c>
       <c r="I118" s="5" t="inlineStr">
         <is>
-          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+          <t>Positive pointsCost requires unassigned offer; redeemed owner/cost immutable; used voucher cannotreactivate. RowVersionconflict409.</t>
         </is>
       </c>
       <c r="J118" s="5" t="inlineStr">
@@ -6389,12 +6413,12 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>body: ComboRequest</t>
+          <t>body: ComboRequest; imageUrl? (HTTP/S,max2048; update null preserves, empty clears)</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200; includes imageUrl nullable</t>
         </is>
       </c>
       <c r="I123" s="5" t="inlineStr">
@@ -6489,7 +6513,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>body: VoucherRequest</t>
+          <t>body: VoucherRequest; pointsCost=0 (0..1000000)</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6499,7 +6523,7 @@
       </c>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>Xem Swagger/controller để biết DTO và điều kiện chi tiết.</t>
+          <t>Positive pointsCost requires unassigned offer; redeemed owner/cost immutable; used voucher cannotreactivate. RowVersionconflict409.</t>
         </is>
       </c>
       <c r="J125" s="5" t="inlineStr">
@@ -6908,8 +6932,558 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>/api/v1/media/images</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Upload ảnh dịch vụ/combo lên Cloudinary</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + SERVICE.WRITE</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>multipart/form-data field file, PNG/JPEG/WebP &lt;=5MiB</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>201 {imageUrl,publicId}</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>400 invalid file;413 oversize;503 unconfigured;502 provider;504 timeout. Save returned imageUrl in service/combo POST/PUT.</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>/api/v1/customers/me/voucher-offers</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Danh sách voucher đổi điểm chưa nhận</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Authenticated customer profile</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>[{id,promotionId,promotionName,discountValue,expiresAt,pointsCost}]</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Codes redacted; unassigned/unredeemed/unused active offers only.403 no profile.</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>/api/v1/customers/me/vouchers/{id}/redeem</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Đổi điểm lấy một mã voucher</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Authenticated customer profile</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>No body</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>200 {voucherId,code,pointsSpent,remainingPoints}</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Atomic balance/ownership/ledger;400 insufficient;403 no profile;404 invalid;409 claimed/concurrent. No double charge on invoice use.</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Đã triển khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>/api/v1/reviews/management</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Management list and filters</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REVIEW.MODERATE</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>serviceId?, from?, to?, stars? (1..5), status? (HienThi/ChoDuyet/An), page=1,pageSize=20 (max100)</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>200 {items,totalCount,averageRating,page,pageSize}</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Includes hidden/pending, customer/service/combo details and saved reply. Excludes soft-deleted. Date boundaries inclusive; use explicit date-time. SQL11.</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>/api/v1/reviews/{id}/reply</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Create or replace staff reply</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REVIEW.MODERATE</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>JSON {reply: string (1..2000, nonblank)}</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Reply saved in database, returned by public visible review list. Deleted/missing404; concurrency409. No automatic push/email. SQL11.</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Reviews</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>/api/v1/reviews/{id}</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Soft-delete violating review</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REVIEW.MODERATE</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Preserves original review/invoice uniqueness and hasReviewed; public/pending/management exclude deleted. Cannot revive via moderation. Missing/deleted404; concurrent409. SQL11.</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>/api/v1/reports/appointment-summary</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Appointment counts by period/status</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>groupBy=day|week|month|status; from?,to?,status?,staffId?,serviceId?,comboId?,categoryId?,search?</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>{totalCount,items:[{periodStart,status,count}]}</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Date range [from,to); Monday weeks; appointment time. Max100000 source rows; overflow400.</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>/api/v1/reports/orders</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Search and paginate service invoices</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>from?,to?,status?,staffId?,serviceId?,comboId?,categoryId?,search?,page=1,pageSize=20 (max100)</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>{totalCount,paidRevenue,page,pageSize,items}</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Invoice creation dates; counts all matching statuses, paidRevenue only settled invoices. Item gross/net distinguished.</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>/api/v1/reports/order-summary</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Invoice counts by day/week/month/quarter/year</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>groupBy=day|week|month|quarter|year; invoice filters</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>{totalCount,paidRevenue,items:[{periodStart,invoiceCount,paidInvoiceCount,unpaidInvoiceCount,paidRevenue}]}</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Defaults groupBy month. Date range [from,to); no partial truncation. Not a payment settlement-date cashflow report.</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>/api/v1/reports/order-breakdown</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Invoice breakdown by service/combo/staff/category</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>groupBy=service|combo|staff|category; invoice filters</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>{totalCount,paidRevenue,metric,items}</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Staff: invoiceNet once per invoice. Service/combo/category: lineGrossBeforeDiscount, no invented net allocation; combos category bucket comboUnallocated. Direct-service/category filters exclude combo components.</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>/api/v1/reports/new-customers</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>New customer counts by creation period</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>groupBy=day|week|month|quarter|year; from?,to?,search?</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>{totalCount,unknownHistoricalCount,items:[{periodStart,count}]}</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>SQL12 adds nullable CreatedAt default for future registrations. Existing unknown dates remain NULL and excluded from period counts, reported separately. Nonapplicable filters400. SQL12 prepared, not applied locally: SSPI blocked live verification.</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J133"/>
+  <autoFilter ref="A1:J136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6920,7 +7494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18" customWidth="1" style="4" min="1" max="1"/>
@@ -7299,6 +7873,40 @@
       <c r="C22" t="inlineStr">
         <is>
           <t>Per-account read receipts; shared broadcast remains unread for other customers</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>UploadImageResponse</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>imageUrl, publicId</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>POST /media/images</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Voucher point exchange</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>pointsCost,redeemedAt,usedAt; ledger voucherId</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>customers/me/voucher-offers; customers/me/vouchers/{id}/redeem</t>
         </is>
       </c>
     </row>
@@ -7313,7 +7921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="13" customWidth="1" style="4" min="1" max="1"/>
@@ -7478,6 +8086,18 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cloudinary/reminders/points (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SQL07..10 additive; images storedasURL; reminder60minutes/dedup; pointsCostexchangeatomic; 28tables unchanged. ShortWebhandoff BAO_CAO_5_CHUC_NANG_WEB.md.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(api): Add prepaid service package lifecycle
Track purchased service sessions, payment receipts and booking reservations.
Consume sessions on completion and retain zero-value receipts for reviews.

Add SQL13 and Vietnamese integration guidance for Web and Flutter.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/KLCN021_API_Catalog.xlsx
+++ b/KLCN021_API_Catalog.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J144"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" style="4" min="1" max="1"/>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Transactions include invoiceId/voucherId links;404 missing;400 invalidpagination.</t>
+          <t>Transactions include invoiceId/voucherId links;404 missing;400 invalidpagination. Transactions append customerPackageId for prepaid purchase reward source.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>appointmentAt, items[{serviceId, comboId?, expectedPrice}], note?, customerId?, staffId?</t>
+          <t>appointmentAt, items[{serviceId, comboId?, expectedPrice}], note?, customerId?, staffId?; customerPackageId? (purchased package ID)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Catalog-derived expectedPrice; complete active combo composition/date required. Management also APPOINTMENT.WRITE. Invalid service/combo/shift400; overlap409.</t>
+          <t>Catalog-derived expectedPrice; complete active combo composition/date required. Management also APPOINTMENT.WRITE. Invalid service/combo/shift400; overlap409. Package-funded all-covered ordinary services only; reserved atomically; response customerPackageId/fundingSource.</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -7479,6 +7479,606 @@
       <c r="J144" t="inlineStr">
         <is>
           <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>List active service packages</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>ServicePackage[] with items[{id,servicePackageId,serviceId,sessions}]</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Active catalog only; includeInactive=true400.</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/{id}</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Get active package detail</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>ServicePackage with items</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Inactive or missing404.</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/management</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Manage complete package catalog</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + SERVICE.WRITE</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>ServicePackage[] with items</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Includes inactive.</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Create package catalog entry</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + SERVICE.WRITE</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>{name,price,validityDays,items:[{serviceId,sessions}],active=true,imageUrl?}</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>201 ServicePackage</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>No duplicate services;1..100items,1..10000sessions,price0.01..1e9 max2decimals,validity1..3650days. SQL13.</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/{id}</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Update or deactivate package</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + SERVICE.WRITE</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Full ServicePackageRequest</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>200 ServicePackage</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Paid purchase snapshots unchanged; Active=false stops new sales, not existing entitlements. Omitted/null image keeps, empty clears.409concurrency.</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/purchases</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Create immutable package purchase snapshot</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Customer owner; management + CUSTOMER.WRITE</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>{packageId,customerId?}</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>201 CustomerPackageView Pending</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Management requires customerId; customer cannot buy for another. Pending available0.</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/purchases/{id}/pay</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Confirm full package payment</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + PAYMENT.WRITE</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>{method: TienMat|ChuyenKhoan|The}</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>200 CustomerPackageView Paid</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Server snapshotprice; one payment, starts expiry, earns floor(price/10000) points once;409retry/conflict. Manual received-payment record, not bank gateway.</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/mine</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>View own packages and session balances</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Authenticated customer profile</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>CustomerPackageView[]</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Per-service granted/reserved/used/remaining/available; expiry or unpaid availability0.</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/customers/{customerId}</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>View customer purchased packages</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + CUSTOMER.READ</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>customerId</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>CustomerPackageView[]</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Purchase snapshots retained after catalog edits.</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/purchases/{id}</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>View package and usage history</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Customer owner; management + CUSTOMER.READ</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>{package:CustomerPackageView,history:[{id,customerPackageItemId,appointmentId,quantity,status,createdAt,settledAt}]}</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>History Reserved/Consumed/Released. Other customer403.</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/purchases/{id}</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Cancel pending package purchase</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Customer owner; management + CUSTOMER.WRITE</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Paid package cannot cancel/refund here409.</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>ServicePackages</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>/api/v1/service-packages/sales</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Report received package purchase income</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Admin/Manager/Reception + REPORT.READ</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>from,to required [from,to), max366days</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>{from,to,count,revenue,items:[{id,customerId,name,price,paidAt,paymentMethod}]}</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>PaidAt basis, separate ordinary invoice revenue; max10000receipts else400.</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Implemented; SQL-backed HTTP smoke verified</t>
         </is>
       </c>
     </row>
@@ -7494,7 +8094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18" customWidth="1" style="4" min="1" max="1"/>
@@ -7907,6 +8507,23 @@
       <c r="C24" t="inlineStr">
         <is>
           <t>customers/me/voucher-offers; customers/me/vouchers/{id}/redeem</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ServicePackage/CustomerPackage</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SQL13:5 package tables</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Catalog plus purchase snapshot,per-service entitlements and usage history. Remaining=granted-used;available=remaining-reserved only paid/unexpired.</t>
         </is>
       </c>
     </row>
@@ -7921,7 +8538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="13" customWidth="1" style="4" min="1" max="1"/>
@@ -8098,6 +8715,18 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Prepaid package revenue</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Package receipt records income once; redemption auto paid zero invoice for reviews, no second points/payment. See HUONG_DAN_GOI_DICH_VU.md. Migrations applied by user; SQL-backed HTTP checks pass, SQL write concurrency unverified.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>